<commit_message>
analysis complete and 37 members failed
</commit_message>
<xml_diff>
--- a/drg/for analysis/results/interpolation.xlsx
+++ b/drg/for analysis/results/interpolation.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\drg\for analysis\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\drg\for analysis\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F915A3-4620-4231-B3C6-3BD4353512E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,8 +35,49 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+  <si>
+    <t>Wall type</t>
+  </si>
+  <si>
+    <t>Breadth (m)</t>
+  </si>
+  <si>
+    <t>Height (m)</t>
+  </si>
+  <si>
+    <t>Unit weight (KN/m2)</t>
+  </si>
+  <si>
+    <t>Load Intensity</t>
+  </si>
+  <si>
+    <t>Without opening</t>
+  </si>
+  <si>
+    <t>With 30% Opening</t>
+  </si>
+  <si>
+    <t>9" wall</t>
+  </si>
+  <si>
+    <t>upto beam</t>
+  </si>
+  <si>
+    <t>upto slab</t>
+  </si>
+  <si>
+    <t>4" wall</t>
+  </si>
+  <si>
+    <t>parapet wall</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -46,15 +87,39 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -62,12 +127,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -347,11 +441,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="C2:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C2">
         <v>0.5</v>
       </c>
@@ -359,7 +453,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C3">
         <v>0.66700000000000004</v>
       </c>
@@ -368,7 +462,7 @@
         <v>1.0834999999999999</v>
       </c>
     </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.3">
       <c r="C4">
         <v>2.5</v>
       </c>
@@ -379,4 +473,205 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0.23</v>
+      </c>
+      <c r="C4" s="6">
+        <v>2.3875999999999999</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="E4" s="6">
+        <v>19.2</v>
+      </c>
+      <c r="F4" s="6">
+        <f>B4*C4*E4</f>
+        <v>10.543641599999999</v>
+      </c>
+      <c r="G4" s="6">
+        <f>B4*D4*E4</f>
+        <v>11.553139200000002</v>
+      </c>
+      <c r="H4" s="6">
+        <f>70%*F4</f>
+        <v>7.3805491199999986</v>
+      </c>
+      <c r="I4" s="6">
+        <f>70%*G4</f>
+        <v>8.0871974400000006</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="7">
+        <v>0.115</v>
+      </c>
+      <c r="C6" s="7">
+        <v>2.3875999999999999</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2.6162000000000001</v>
+      </c>
+      <c r="E6" s="7">
+        <v>19.2</v>
+      </c>
+      <c r="F6" s="7">
+        <f>B6*C6*E6</f>
+        <v>5.2718207999999995</v>
+      </c>
+      <c r="G6" s="7">
+        <f>B6*D6*E6</f>
+        <v>5.7765696000000011</v>
+      </c>
+      <c r="H6" s="7">
+        <f>70%*F6</f>
+        <v>3.6902745599999993</v>
+      </c>
+      <c r="I6" s="7">
+        <f>70%*G6</f>
+        <v>4.0435987200000003</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="5">
+        <v>0.115</v>
+      </c>
+      <c r="C8" s="8">
+        <v>1.0668</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="5">
+        <v>19.2</v>
+      </c>
+      <c r="F8" s="8">
+        <f>B8*C8*E8</f>
+        <v>2.3554944</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>